<commit_message>
fix(catalog): prioritize local Excel path for seamless serverless deployment
</commit_message>
<xml_diff>
--- a/JM_Dishes_Mapping_Expanded_SuperAdmin.xlsx
+++ b/JM_Dishes_Mapping_Expanded_SuperAdmin.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Super Admin - AP New Dishes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final 50 AP Dishes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Super Admin - AP New Dishes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +30,12 @@
       <b val="1"/>
       <color rgb="001F2937"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +46,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2E7EB"/>
         <bgColor rgb="00F2E7EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +67,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,8 +438,3354 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="52" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>SORT ORDER</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>NAME (EN) *</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Telugu Name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>CLUSTER</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>EMOJI</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>MEAL TABS</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FOOD GROUPS (MDD-W)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Vegetarian</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Contains Egg</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>IMAGE URL (Direct for Super Admin)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Backup Image URL</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Saved Local File Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Thotakura Vepudu / Kura (Amaranth)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>తోటకూర వేపుడు / కూర</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Leafy Green Curries</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>🥬</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/67/03/4f/67034f5c16e5a93e968a171e3a1e7005.jpg</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Thotakura Vepudu / Kura (Amaranth)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\01_Thotakura_Vepudu_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Palakura Kura / Vepudu (Spinach)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>పాలకూర కూర / వేపుడు</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Leafy Green Curries</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>🥬</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/c8/16/81/c816810bbaf03dfc3b7f22be96a1ccef.jpg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Palakura%20Kura%20/%20Vepudu%20%28Spinach%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\02_Palakura_Kura_Vepudu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gongura Kura / Pulusu (Sorrel Leaves)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>గోంగూర కూర / పులుసు</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Leafy Green Curries</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>🌿</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/f4/b1/cc/f4b1cc054c32209879e5a64fe9b3c516.jpg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Gongura Kura / Pulusu (Sorrel Leaves)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\03_Gongura_Kura_Pulusu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Menthi Kura Vepudu / Kura (Fenugreek)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>మెంతికూర వేపుడు / కూర</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Leafy Green Curries</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>🌿</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://blogger.googleusercontent.com/img/b/R29vZ2xl/AVvXsEjXLTJ9wsm7MzOwsgxmlM7CFGKns25pouV5CVrZKcDItAoga1GuOdESEBK_oZ8sh2w2L1ggnMVDhwc2cOuComjCJPDcb4ckI11pD-j-scjXqHP0rP3NBv8nEsHLEVNvxckbMzD2QUi0gcQ/s1600/IMG_8574.JPG</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Menthi%20Kura%20Vepudu%20/%20Kura%20%28Fenugreek%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\04_Menthi_Kura_Vepudu_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Munagaku Vepudu / Kura (Drumstick Leaves)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>మునగాకు వేపుడు / కూర</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Leafy Green Curries</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>🌿</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/b3/0b/b5/b30bb56ae7a6b6dcabec0e943c384da9.jpg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/db/31/7d/db317d1c206226e4d27e3529c20bf42b.jpg</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\05_Munagaku_Vepudu_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Palakura Pappu (Spinach Dal)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>పాలకూర పప్పు</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/9f/25/f8/9f25f8d8ca39f213b1ef3a603c93c414.jpg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/e8/6b/a4/e86ba4ab6c0b149128c65cb0d0f22211.jpg</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\06_Palakura_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Thotakura Pappu (Amaranth Dal)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>తోటకూర పప్పు</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://everydaynourishingfoods.com/wp-content/uploads/2021/02/thotakura-pappu-featured-image-1024x1024.jpg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Thotakura%20Pappu%20%28Amaranth%20Dal%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\07_Thotakura_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gongura Pappu (Sorrel Leaves Dal)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>గోంగూర పప్పు</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.indianhealthyrecipes.com/wp-content/uploads/2022/08/gongura-pappu-recipe.webp</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Gongura%20Pappu%20%28Sorrel%20Leaves%20Dal%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\08_Gongura_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Menthi Kura Pappu (Fenugreek Dal)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>మెంతికూర పప్పు</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.indianhealthyrecipes.com/wp-content/uploads/2020/01/methi-dal.jpg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Menthi%20Kura%20Pappu%20%28Fenugreek%20Dal%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\09_Menthi_Kura_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Chukkakura Pappu (Green Sorrel Dal)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>చుక్కకూర పప్పు</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.sandyathome.com/wp-content/uploads/2025/06/pulicha-keerai-pappu-traditional-recipe.jpg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Chukkakura%20Pappu%20%28Green%20Sorrel%20Dal%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\10_Chukkakura_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dosakaya Pappu (Yellow Cucumber Dal)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>దోసకాయ పప్పు</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://www.subbuskitchen.com/wp-content/uploads/2021/10/dosakaya-pappu_web4.jpg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Dosakaya%20Pappu%20%28Yellow%20Cucumber%20Dal%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\11_Dosakaya_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sorakaya Pappu (Bottle Gourd Dal)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>సొరకాయ పప్పు</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://subbucooks.com/wp-content/uploads/2020/02/IMG_5530-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Sorakaya%20Pappu%20%28Bottle%20Gourd%20Dal%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\12_Sorakaya_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mamidikaya Pappu (Raw Mango Dal)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>మామిడికాయ పప్పు</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/60/f7/27/60f727956329c693316141ccb957a9c5.jpg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://blogger.googleusercontent.com/img/b/R29vZ2xl/AVvXsEgggMO52-kWRNbbYBFYBW1UUwsK3ejiw3hvFI3dEthhjRv5rcIOo-FSz5svjCesBLsFiUvebYss7EA4CxS1JD2LttQN-5wCoe1uozvrhOa8oLLfxSGnoRVhH2cBghkVBr_yjbWKLQ1EjO4/s1600/Pachi+Mamidikaya+Pappu+11.JPG</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\13_Mamidikaya_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Beerakaya Pappu (Ridge Gourd Dal)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>బీరకాయ పప్పు</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Dals &amp; Pappu</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://www.indianhealthyrecipes.com/wp-content/uploads/2022/07/beerakaya-pappu-recipe.webp</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Beerakaya%20Pappu%20%28Ridge%20Gourd%20Dal%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\14_Beerakaya_Pappu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vankaya Kura / Gutti Vankaya (Brinjal)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>వంకాయ కూర / గుత్తి వంకాయ</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>🍆</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables, G3 Nuts and seeds</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/b8/42/75/b842758dcb127989e1f4c2884e8eaaf3.jpg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/b8/42/75/b842758dcb127989e1f4c2884e8eaaf3.jpg</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\15_Vankaya_Kura_Gutti_Vankaya.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bendakaya Vepudu / Pulusu (Ladies Finger)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>బెండకాయ వేపుడు / పులుసు</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>🥘</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://www.sandyathome.com/wp-content/uploads/2016/11/IMG_4887.jpg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Bendakaya%20Vepudu%20/%20Pulusu%20%28Ladies%20Finger%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\16_Bendakaya_Vepudu_Pulusu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bangaladumpa / Aloo Vepudu (Potato Fry)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>బంగాళాదుంప వేపుడు</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>🥔</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Breakfast, Meals</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>G1 Grains, roots &amp; tubers, G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/62/09/ff/6209ff8c8178bf5e7171e1a1aca81f34.jpg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Bangaladumpa%20/%20Aloo%20Vepudu%20%28Potato%20Fry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\17_Bangaladumpa_Aloo_Vepudu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dondakaya Vepudu (Ivy Gourd Fry)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>దొండకాయ వేపుడు</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://www.subbuskitchen.com/wp-content/uploads/2022/02/kovakkai-fry-web1.jpg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Dondakaya%20Vepudu%20%28Ivy%20Gourd%20Fry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\18_Dondakaya_Vepudu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Beerakaya Kura (Ridge Gourd Curry)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>బీరకాయ కూర</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://www.masalakorb.com/wp-content/uploads/2017/11/Beerakaya-Palu-Curry-V2.jpg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Beerakaya%20Kura%20%28Ridge%20Gourd%20Curry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\19_Beerakaya_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Sorakaya / Anapakaya Kura (Bottle Gourd)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>సొరకాయ కూర</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://blogger.googleusercontent.com/img/b/R29vZ2xl/AVvXsEhquNxQPayZ2MC7esGEsjm7DypSxLglpU7HayP8vfJO3hx73HimySSVW3x7IT4nLlmPZUg6Lx3DVxAzphe499tKQ2qPVaPyu3Qwe3gQk6Zgxz-rHfCSXRlFODMOaSdIS_iyxgFk3HWaMg2YNp3yrJ1ihw0NmqdOT3mL_dK0cwMyAHKE5vZQaltn3TR6/s1600/Sorakaya_AvaKura.jpg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Sorakaya%20/%20Anapakaya%20Kura%20%28Bottle%20Gourd%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\20_Sorakaya_Anapakaya_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kakarakaya Vepudu / Pulusu (Bitter Gourd)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>కాకరకాయ వేపుడు / పులుసు</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://vismaifood.com/storage/app/uploads/public/27e/c69/cb9/thumb__700_0_0_0_auto.jpg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Kakarakaya%20Vepudu%20/%20Pulusu%20%28Bitter%20Gourd%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\21_Kakarakaya_Vepudu_Pulusu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cabbage Vepudu (Cabbage Stir-Fry)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>క్యాబేజీ వేపుడు</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>🥬</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://www.indianhealthyrecipes.com/wp-content/uploads/2022/02/cabbage-poriyal.jpg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Cabbage%20Vepudu%20%28Cabbage%20Stir-Fry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\22_Cabbage_Vepudu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Cauliflower Kura (Cauliflower Curry)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>కాలిఫ్లవర్ కూర</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>🥦</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/aa/4d/02/aa4d027a50201577c7a2ad2496905458.jpg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Cauliflower Kura (Cauliflower Curry)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\23_Cauliflower_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Beans Vepudu (French Beans Stir-Fry)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>బీన్స్ వేపుడు</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>🫛</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/55/f5/f7/55f5f7c1f6bf796f2f7b1a5f2922033c.jpg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Beans%20Vepudu%20%28French%20Beans%20Stir-Fry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\24_Beans_Vepudu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Chikkudukaya Kura (Broad Beans Curry)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>చిక్కుడుకాయ కూర</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>🫛</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables, G2 Pulses (beans, peas, lentils)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://cravingsphere.com/imageassets/a851a0bc-3666-4d66-8c12-d713752f9008.png</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Chikkudukaya%20Kura%20%28Broad%20Beans%20Curry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\25_Chikkudukaya_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Goruchikkudu Kura (Cluster Beans Curry)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>గోరుచిక్కుడు కూర</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>🫛</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://www.indianhealthyrecipes.com/wp-content/uploads/2022/10/cluster-beans-goruchikkudu-guar-beans.webp</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Goruchikkudu%20Kura%20%28Cluster%20Beans%20Curry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\26_Goruchikkudu_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Dosakaya Kura / Mukkala Pulusu</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>దోసకాయ కూర / పులుసు</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://www.fatrainbow.com/wp-content/uploads/2020/10/Dosakaya-tomato-kura-1-683x1024.jpg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Dosakaya%20Kura%20/%20Mukkala%20Pulusu&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\27_Dosakaya_Kura_Mukkala_Pulusu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Munakkaya Kura / Pulusu (Drumstick Curry)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>మునక్కాయ కూర / పులుసు</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>🥘</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://vismaifood.com/storage/app/uploads/public/423/afb/849/thumb__1200_0_0_0_auto.jpg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Munakkaya%20Kura%20/%20Pulusu%20%28Drumstick%20Curry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\28_Munakkaya_Kura_Pulusu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Aratikaya Vepudu / Kura (Raw Banana)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>అరటికాయ వేపుడు / కూర</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>🍌</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>G1 Grains, roots &amp; tubers</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/0a/71/27/0a7127aee202fb450a6ae5b46600cee3.jpg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Aratikaya%20Vepudu%20/%20Kura%20%28Raw%20Banana%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\29_Aratikaya_Vepudu_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Chamadumpa Pulusu / Vepudu (Colocasia)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>చామదుంప పులుసు / వేపుడు</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>🥔</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>G1 Grains, roots &amp; tubers, G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>http://3.bp.blogspot.com/-W66Pjq7WwUM/U7OTZGq_wbI/AAAAAAAAFQA/LsMGfv3NoIY/s1600/Colocasia+Tomato+Curry+ChamaDumpa+Pulusu+in+Telugu+with+English+Sub+Titles.mp4_snapshot_00.16_[2014.07.01_12.24.42].jpg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Chamadumpa%20Pulusu%20/%20Vepudu%20%28Colocasia%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\30_Chamadumpa_Pulusu_Vepudu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Potlakaya Kura (Snake Gourd Curry)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>పొట్లకాయ కూర</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables, G4 Dairy</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://4.bp.blogspot.com/-1xVJmiCkAFU/UA4Bo486lTI/AAAAAAAAIHc/y0O7kxfe2JI/s1600/DSC_0385.jpg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Potlakaya%20Kura%20%28Snake%20Gourd%20Curry%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\31_Potlakaya_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Meal Maker / Soya Chunks Kura</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>మీల్ మేకర్ / సోయా కూర</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>🥘</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/53/d7/06/53d70679cc2eb16f3f25e4eadcd80d77.jpg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/b8/f0/70/b8f070c6268b66c4299aa0019a38bdb2.jpg</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\32_Meal_Maker_Soya_Chunks_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Senagala Kura (Brown Chickpea Curry)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>శనగల కూర</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>🥘</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Breakfast, Meals</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils), G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/83/43/0c/83430cbc5a7420c116a8593bc60127be.jpg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Senagala Kura (Brown Chickpea Curry)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\33_Senagala_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Majjiga Pulusu / Majjiga Charu</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>మజ్జిగ పులుసు</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Vegetable Curries</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>🥣</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>G4 Dairy, G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/b0/ba/6e/b0ba6ebd2ea2f2df719f37fa5dbf3c66.jpg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Majjiga Pulusu / Majjiga Charu&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\34_Majjiga_Pulusu_Majjiga_Charu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Palli Pachadi (Peanut Chutney)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>పల్లీ పచ్చడి</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Chutneys &amp; Podis</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>🥜</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Breakfast, Meals</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>G3 Nuts and seeds</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/70/9d/a2/709da2b9dacb24e90eb3989302abe020.jpg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Palli Pachadi (Peanut Chutney)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\35_Palli_Pachadi.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Kobbari Pachadi (Coconut Chutney)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>కొబ్బరి పచ్చడి</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Chutneys &amp; Podis</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>🥥</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Breakfast, Meals</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>G3 Nuts and seeds</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/71/d5/d1/71d5d1cf724742b1c2704b1c5605c6f0.jpg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/ca/25/3d/ca253d51d3e376c5e55f52a2440a53d9.jpg</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\36_Kobbari_Pachadi.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Tomato Pachadi / Roti Pachadi</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>టమాటా పచ్చడి / రోటి పచ్చడి</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Chutneys &amp; Podis</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>🍅</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Breakfast, Meals</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://www.indianhealthyrecipes.com/wp-content/uploads/2022/08/tomato-pachadi-recipe.jpg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Tomato%20Pachadi%20/%20Roti%20Pachadi&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\37_Tomato_Pachadi_Roti_Pachadi.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Dosakaya Pachadi (Yellow Cucumber Chutney)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>దోసకాయ పచ్చడి</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Chutneys &amp; Podis</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://www.cookshideout.com/wp-content/uploads/2013/09/Dosakaya-Pachadi-FI.jpg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Dosakaya%20Pachadi%20%28Yellow%20Cucumber%20Chutney%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\38_Dosakaya_Pachadi.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Guddu Porutu / Egg Bhurji (Scrambled Egg)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>గుడ్డు పొరుటు / ఎగ్ బుర్జీ</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Eggs, Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>🍳</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>G6 Eggs, G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://www.masalakorb.com/wp-content/uploads/2020/07/Egg-Bhurji-Masala-Egg-Porutu-Andhra-Style-V2-683x1024.jpg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Guddu%20Porutu%20/%20Egg%20Bhurji%20%28Scrambled%20Egg%29&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\39_Guddu_Porutu_Egg_Bhurji.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Egg Curry (Guddu Kura / Guddu Pulusu)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>గుడ్డు కూర / పులుసు</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Eggs, Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>🥚</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>G6 Eggs, G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/e2/8d/b3/e28db3b9af80175f458b97846bf129b1.jpg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Egg Curry (Guddu Kura / Guddu Pulusu)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\40_Egg_Curry.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Natukodi Pulusu (Country Chicken Curry)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>నాటుకోడి పులుసు</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Eggs, Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>🍗</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>G5 Meat, poultry and fish, G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/0d/a6/43/0da6433a3084a354bfd2abb804f20942.png</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Natukodi Pulusu (Country Chicken Curry)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\41_Natukodi_Pulusu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Gongura Chicken</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>గోంగూర చికెన్</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Eggs, Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>🍗</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>G5 Meat, poultry and fish, G7 Dark green leafy vegetables</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/a6/b2/64/a6b2647dd407ea0256f0842dc93b3b03.jpg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Gongura%20Chicken&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\42_Gongura_Chicken.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Endu Chepalu Kura (Dry Fish Curry)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ఎండు చేపల కూర</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Eggs, Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>🐟</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Meals</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>G5 Meat, poultry and fish, G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/44/26/f3/4426f3e21005c674111cfee1bfbb1f76.jpg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Endu Chepalu Kura (Dry Fish Curry)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\43_Endu_Chepalu_Kura.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Carrot (Raw / Slices / Salad)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>పచ్చి క్యారెట్</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Vegetables &amp; Salads</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>🥕</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Snacks, Meals</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>G4 Vitamin A-rich vegetables &amp; fruits</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/0a/11/d0/0a11d076f6a66ac8ba0aeb6d61df5858.jpg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Carrot (Raw / Slices / Salad)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\44_Carrot.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Cucumber / Keera Dosakaya (Raw / Salad)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>కీరదోస / కీరకాయ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Vegetables &amp; Salads</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>🥒</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Snacks, Meals</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>G9 Other vegetables</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/57/5c/cc/575ccc4ca5459889951ae5c76376e9b4.jpg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Cucumber / Keera Dosakaya (Raw / Salad)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\45_Cucumber_Keera_Dosakaya.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Walnuts (Akrotu)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>వాల్‌నట్స్ / ఆక్రోట్</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>🥜</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Snacks, Breakfast</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>G3 Nuts and seeds</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/4a/69/b5/4a69b53057ba000cac286346435d4be5.jpg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/bb/7b/5c/bb7b5ce0bd844aa9f0d18c1f1154f288.jpg</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\46_Walnuts.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Dry Fruit Laddu (Dates &amp; Nuts Laddu)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>డ్రై ఫ్రూట్ లడ్డూ (ఖర్జూరం లడ్డూ)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Snacks &amp; Sweets</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>🧆</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>G3 Nuts and seeds, G5 Other fruits</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/a4/be/ba/a4beba8c7722a9b65de806067fbed2d8.jpg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Dry Fruit Laddu (Dates &amp; Nuts Laddu)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\47_Dry_Fruit_Laddu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Guggillu (Boiled Seasoned Chickpeas)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>గుగ్గిళ్ళు</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Snacks &amp; Sweets</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>🫘</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Fruits/Nuts, Snacks</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>G2 Pulses (beans, peas, lentils)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/5d/3b/3a/5d3b3aaa5039830efecac969d8187a8d.jpg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://tse2.mm.bing.net/th?q=Guggillu (Boiled Seasoned Chickpeas)&amp;w=800&amp;h=800&amp;c=7</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\48_Guggillu.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Ragi Malt (Finger Millet Health Drink)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>రాగి మాల్ట్</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Beverages &amp; Millets</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>🥛</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Breakfast, Snacks</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>G1 Grains, roots &amp; tubers, G7 Dairy</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/25/03/19/25031942531a497fa13fe8bda4f90d34.jpg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/77/34/1f/77341ffc47913d23370a0136ff590570.jpg</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\49_Ragi_Malt.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Coconut Water (Kobbari Bondam)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>కొబ్బరి బొండం</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>🥥</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Fruits/Nuts, Snacks</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>G10 Other fruits</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/736x/d9/02/2c/d9022c0da0d195e93ac500586bf0dd37.jpg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>https://i.pinimg.com/originals/89/6c/03/896c03eba3d56d3f7e0c9d143d4b6fee.jpg</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>C:\Users\rinit\Downloads\Jm_app_asha_visit_sample\AP_50_Dish_Images\All_50_Dishes\50_Coconut_Water.jpg</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>

</xml_diff>